<commit_message>
further enhancement in admin UI
</commit_message>
<xml_diff>
--- a/apps/web/public/templates/question-import-template.xlsx
+++ b/apps/web/public/templates/question-import-template.xlsx
@@ -1,109 +1,43 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
-  <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sudjangr\Downloads\technical-pilot-lms\apps\web\public\templates\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF590B35-BE27-4D8F-8D47-3C8E6CF88136}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
-  <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
-  </bookViews>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <workbookPr codeName="ThisWorkbook"/>
   <sheets>
     <sheet name="Questions" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="25">
-  <si>
-    <t>question_number</t>
-  </si>
-  <si>
-    <t>question_text</t>
-  </si>
-  <si>
-    <t>question_type</t>
-  </si>
-  <si>
-    <t>points</t>
-  </si>
-  <si>
-    <t>explanation</t>
-  </si>
-  <si>
-    <t>What is the capital of France?</t>
-  </si>
-  <si>
-    <t>mcq</t>
-  </si>
-  <si>
-    <t>Paris has been the capital since the 12th century.</t>
-  </si>
-  <si>
-    <t>Paris</t>
-  </si>
-  <si>
-    <t>Which of these are prime numbers?</t>
-  </si>
-  <si>
-    <t>msq</t>
-  </si>
-  <si>
-    <t>2, 3 and 5 are prime; 4 is not (divisible by 2).</t>
-  </si>
-  <si>
-    <t>text</t>
-  </si>
-  <si>
-    <t>option_A</t>
-  </si>
-  <si>
-    <t>option_B</t>
-  </si>
-  <si>
-    <t>option_C</t>
-  </si>
-  <si>
-    <t>option_D</t>
-  </si>
-  <si>
-    <t>answer</t>
-  </si>
-  <si>
-    <t>Delhi</t>
-  </si>
-  <si>
-    <t>New York</t>
-  </si>
-  <si>
-    <t>All of above</t>
-  </si>
-  <si>
-    <t>C</t>
-  </si>
-  <si>
-    <t>D</t>
-  </si>
-  <si>
-    <t>What is 2+2=?</t>
-  </si>
-  <si>
-    <t>2+2 = 4</t>
-  </si>
-</sst>
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
+  <numFmts count="1">
+    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
+  </numFmts>
+  <fonts count="1">
     <font>
-      <sz val="11"/>
+      <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -131,21 +65,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
 </styleSheet>
 </file>
 
@@ -224,6 +150,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -258,6 +185,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -292,20 +220,16 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:shade val="51000"/>
+                <a:tint val="100000"/>
+                <a:shade val="100000"/>
                 <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="80000">
-              <a:schemeClr val="phClr">
-                <a:shade val="93000"/>
-                <a:satMod val="130000"/>
-              </a:schemeClr>
-            </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="94000"/>
-                <a:satMod val="135000"/>
+                <a:tint val="50000"/>
+                <a:shade val="100000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
@@ -427,142 +351,197 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
+  <a:objectDefaults>
+    <a:spDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="3">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </a:style>
+    </a:spDef>
+    <a:lnDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </a:style>
+    </a:lnDef>
+  </a:objectDefaults>
   <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="16" customWidth="1"/>
-    <col min="2" max="2" width="45" customWidth="1"/>
-    <col min="3" max="3" width="16" customWidth="1"/>
-    <col min="4" max="4" width="8" customWidth="1"/>
-    <col min="5" max="5" width="45" customWidth="1"/>
-    <col min="6" max="6" width="20" customWidth="1"/>
-    <col min="7" max="7" width="12" customWidth="1"/>
-  </cols>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:K4"/>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E1" t="s">
-        <v>14</v>
-      </c>
-      <c r="F1" t="s">
-        <v>15</v>
-      </c>
-      <c r="G1" t="s">
-        <v>16</v>
-      </c>
-      <c r="H1" t="s">
-        <v>17</v>
-      </c>
-      <c r="I1" t="s">
-        <v>3</v>
-      </c>
-      <c r="J1" t="s">
-        <v>4</v>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>question_number</v>
+      </c>
+      <c r="B1" t="str">
+        <v>question_text</v>
+      </c>
+      <c r="C1" t="str">
+        <v>question_type</v>
+      </c>
+      <c r="D1" t="str">
+        <v>option_A</v>
+      </c>
+      <c r="E1" t="str">
+        <v>option_B</v>
+      </c>
+      <c r="F1" t="str">
+        <v>option_C</v>
+      </c>
+      <c r="G1" t="str">
+        <v>option_D</v>
+      </c>
+      <c r="H1" t="str">
+        <v>answer</v>
+      </c>
+      <c r="I1" t="str">
+        <v>points</v>
+      </c>
+      <c r="J1" t="str">
+        <v>explanation</v>
+      </c>
+      <c r="K1" t="str">
+        <v>topic</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="2">
       <c r="A2">
         <v>1</v>
       </c>
-      <c r="B2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D2" t="s">
-        <v>18</v>
-      </c>
-      <c r="E2" t="s">
-        <v>19</v>
-      </c>
-      <c r="F2" t="s">
-        <v>8</v>
-      </c>
-      <c r="G2" t="s">
-        <v>20</v>
-      </c>
-      <c r="H2" t="s">
-        <v>21</v>
+      <c r="B2" t="str">
+        <v>What is the capital of France?</v>
+      </c>
+      <c r="C2" t="str">
+        <v>mcq</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Delhi</v>
+      </c>
+      <c r="E2" t="str">
+        <v>New York</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Paris</v>
+      </c>
+      <c r="G2" t="str">
+        <v>All of above</v>
+      </c>
+      <c r="H2" t="str">
+        <v>C</v>
       </c>
       <c r="I2">
         <v>1</v>
       </c>
-      <c r="J2" t="s">
-        <v>7</v>
+      <c r="J2" t="str">
+        <v>Paris has been the capital since the 12th century.</v>
+      </c>
+      <c r="K2" t="str">
+        <v>Geography</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="3">
       <c r="A3">
         <v>2</v>
       </c>
-      <c r="B3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C3" t="s">
-        <v>10</v>
-      </c>
-      <c r="D3">
+      <c r="B3" t="str">
+        <v>Which of these are prime numbers?</v>
+      </c>
+      <c r="C3" t="str">
+        <v>msq</v>
+      </c>
+      <c r="D3" t="str">
         <v>2</v>
       </c>
-      <c r="E3">
+      <c r="E3" t="str">
         <v>3</v>
       </c>
-      <c r="F3">
+      <c r="F3" t="str">
         <v>5</v>
       </c>
-      <c r="G3" t="s">
-        <v>20</v>
-      </c>
-      <c r="H3" t="s">
-        <v>22</v>
+      <c r="G3" t="str">
+        <v>All of above</v>
+      </c>
+      <c r="H3" t="str">
+        <v>D</v>
       </c>
       <c r="I3">
         <v>1</v>
       </c>
-      <c r="J3" t="s">
-        <v>11</v>
+      <c r="J3" t="str">
+        <v>2, 3 and 5 are prime; 4 is not (divisible by 2).</v>
+      </c>
+      <c r="K3" t="str">
+        <v>Mathematics</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="4">
       <c r="A4">
         <v>3</v>
       </c>
-      <c r="B4" t="s">
-        <v>23</v>
-      </c>
-      <c r="C4" t="s">
-        <v>12</v>
-      </c>
-      <c r="H4">
+      <c r="B4" t="str">
+        <v>What is 2+2=?</v>
+      </c>
+      <c r="C4" t="str">
+        <v>text</v>
+      </c>
+      <c r="D4" t="str">
+        <v/>
+      </c>
+      <c r="E4" t="str">
+        <v/>
+      </c>
+      <c r="F4" t="str">
+        <v/>
+      </c>
+      <c r="G4" t="str">
+        <v/>
+      </c>
+      <c r="H4" t="str">
         <v>4</v>
       </c>
       <c r="I4">
         <v>2</v>
       </c>
-      <c r="J4" t="s">
-        <v>24</v>
+      <c r="J4" t="str">
+        <v>2+2 = 4</v>
+      </c>
+      <c r="K4" t="str">
+        <v>Mathematics</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:K4"/>
+  </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>